<commit_message>
Hosting: require in-person meetings, set call timing, drop old ISBA template
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/files/budget_template.xlsx
+++ b/assets/files/budget_template.xlsx
@@ -714,11 +714,6 @@
       <c r="D19" s="24" t="n">
         <v>6000</v>
       </c>
-      <c r="E19" s="18" t="inlineStr">
-        <is>
-          <t>Including remote transmission if hybrid.</t>
-        </is>
-      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="16">
       <c r="A20" s="19" t="inlineStr">

</xml_diff>